<commit_message>
fix(data): correction to the geometry profile config file
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\Tkinter\production-counting\project\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\production_counting_class\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E87D85B-1814-4175-B9A0-F3CB796D2D98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2597FC29-F889-42B2-B6FA-EAE9FF03FC34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2782,7 +2782,7 @@
         <v>406323</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C175">
         <v>90</v>

</xml_diff>

<commit_message>
fix: add new row for geometry with new set up time
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\production_counting_class\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2597FC29-F889-42B2-B6FA-EAE9FF03FC34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63F7681-DBB4-4D91-8D9B-0F327642E020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="profile_config" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="178">
   <si>
     <t>GP8280</t>
   </si>
@@ -854,7 +854,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C575"/>
+  <dimension ref="A1:C576"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
@@ -6885,7 +6885,7 @@
         <v>149</v>
       </c>
       <c r="B548" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C548">
         <v>110</v>
@@ -6893,7 +6893,7 @@
     </row>
     <row r="549" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A549" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B549" s="1" t="s">
         <v>30</v>
@@ -6907,32 +6907,32 @@
         <v>150</v>
       </c>
       <c r="B550" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C550">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="551" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A551" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B551" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C551">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="552" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A552" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B552" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C552">
-        <v>150</v>
+        <v>60</v>
       </c>
     </row>
     <row r="553" spans="1:3" x14ac:dyDescent="0.25">
@@ -6940,18 +6940,18 @@
         <v>151</v>
       </c>
       <c r="B553" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C553">
-        <v>110</v>
+        <v>150</v>
       </c>
     </row>
     <row r="554" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A554">
-        <v>721014</v>
+      <c r="A554" t="s">
+        <v>151</v>
       </c>
       <c r="B554" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C554">
         <v>110</v>
@@ -6959,24 +6959,24 @@
     </row>
     <row r="555" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A555">
-        <v>721008</v>
+        <v>721014</v>
       </c>
       <c r="B555" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C555">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="556" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A556">
-        <v>721005</v>
+        <v>721008</v>
       </c>
       <c r="B556" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C556">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="557" spans="1:3" x14ac:dyDescent="0.25">
@@ -6984,15 +6984,15 @@
         <v>721005</v>
       </c>
       <c r="B557" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C557">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="558" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A558">
-        <v>721008</v>
+        <v>721005</v>
       </c>
       <c r="B558" s="1" t="s">
         <v>1</v>
@@ -7003,24 +7003,24 @@
     </row>
     <row r="559" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A559">
+        <v>721008</v>
+      </c>
+      <c r="B559" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C559">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="560" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A560">
         <v>721014</v>
       </c>
-      <c r="B559" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C559">
+      <c r="B560" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C560">
         <v>50</v>
-      </c>
-    </row>
-    <row r="560" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A560" t="s">
-        <v>152</v>
-      </c>
-      <c r="B560" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C560">
-        <v>110</v>
       </c>
     </row>
     <row r="561" spans="1:3" x14ac:dyDescent="0.25">
@@ -7028,32 +7028,32 @@
         <v>152</v>
       </c>
       <c r="B561" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C561">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="562" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A562" t="s">
+        <v>152</v>
+      </c>
+      <c r="B562" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C562">
         <v>60</v>
       </c>
     </row>
-    <row r="562" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A562">
+    <row r="563" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A563">
         <v>241040</v>
       </c>
-      <c r="B562" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C562">
+      <c r="B563" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C563">
         <v>120</v>
-      </c>
-    </row>
-    <row r="563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A563">
-        <v>241020</v>
-      </c>
-      <c r="B563" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C563">
-        <v>70</v>
       </c>
     </row>
     <row r="564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7061,43 +7061,43 @@
         <v>241020</v>
       </c>
       <c r="B564" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C564">
-        <v>110</v>
+        <v>70</v>
       </c>
     </row>
     <row r="565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A565">
-        <v>241040</v>
+        <v>241020</v>
       </c>
       <c r="B565" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C565">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A566">
-        <v>601138</v>
+        <v>241040</v>
       </c>
       <c r="B566" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C566">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="567" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A567">
-        <v>601128</v>
+        <v>601138</v>
       </c>
       <c r="B567" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C567">
-        <v>80</v>
+        <v>110</v>
       </c>
     </row>
     <row r="568" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7105,54 +7105,54 @@
         <v>601128</v>
       </c>
       <c r="B568" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C568">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="569" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A569">
+        <v>601128</v>
+      </c>
+      <c r="B569" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C569">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="570" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A570">
         <v>601138</v>
       </c>
-      <c r="B569" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C569">
+      <c r="B570" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C570">
         <v>60</v>
-      </c>
-    </row>
-    <row r="570" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A570" t="s">
-        <v>153</v>
-      </c>
-      <c r="B570" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C570">
-        <v>120</v>
       </c>
     </row>
     <row r="571" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A571" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B571" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C571">
-        <v>70</v>
+        <v>120</v>
       </c>
     </row>
     <row r="572" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A572" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B572" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C572">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="573" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7160,31 +7160,42 @@
         <v>155</v>
       </c>
       <c r="B573" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C573">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="574" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A574" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B574" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C574">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="575" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A575" t="s">
+        <v>154</v>
+      </c>
+      <c r="B575" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C575">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="576" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A576" t="s">
         <v>153</v>
       </c>
-      <c r="B575" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C575">
+      <c r="B576" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C576">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: add missing profiles in the list
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\production_counting_class\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D455729F-15EF-4D93-884A-1EC083006A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE47244-9745-4012-BDB9-8E05B9DB9AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="180">
   <si>
     <t>GP8280</t>
   </si>
@@ -573,6 +573,9 @@
   </si>
   <si>
     <t>GP1401</t>
+  </si>
+  <si>
+    <t>GO2230</t>
   </si>
 </sst>
 </file>
@@ -857,7 +860,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C579"/>
+  <dimension ref="A1:C580"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
@@ -2136,7 +2139,7 @@
         <v>39</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C116">
         <v>120</v>
@@ -3265,14 +3268,14 @@
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A219">
-        <v>416272</v>
+      <c r="A219" t="s">
+        <v>179</v>
       </c>
       <c r="B219" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C219">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
@@ -3280,21 +3283,21 @@
         <v>416272</v>
       </c>
       <c r="B220" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C220">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221">
-        <v>666000</v>
+        <v>416272</v>
       </c>
       <c r="B221" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C221">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
@@ -3302,29 +3305,29 @@
         <v>666000</v>
       </c>
       <c r="B222" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C222">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A223">
+        <v>666000</v>
+      </c>
+      <c r="B223" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C223">
         <v>130</v>
-      </c>
-    </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A223" t="s">
-        <v>61</v>
-      </c>
-      <c r="B223" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C223">
-        <v>90</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C224">
         <v>90</v>
@@ -3335,21 +3338,21 @@
         <v>62</v>
       </c>
       <c r="B225" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C225">
         <v>90</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A226">
-        <v>406005</v>
+      <c r="A226" t="s">
+        <v>62</v>
       </c>
       <c r="B226" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C226">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
@@ -3357,92 +3360,92 @@
         <v>406005</v>
       </c>
       <c r="B227" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C227">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228">
-        <v>716020</v>
+        <v>406005</v>
       </c>
       <c r="B228" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C228">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229">
+        <v>716020</v>
+      </c>
+      <c r="B229" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C229">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A230">
         <v>736323</v>
       </c>
-      <c r="B229" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C229">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A230" t="s">
-        <v>63</v>
-      </c>
       <c r="B230" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C230">
         <v>120</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A231">
+      <c r="A231" t="s">
+        <v>63</v>
+      </c>
+      <c r="B231" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C231">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A232">
         <v>416112</v>
       </c>
-      <c r="B231" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C231">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A232" t="s">
+      <c r="B232" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C232">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
         <v>64</v>
       </c>
-      <c r="B232" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C232">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A233">
+      <c r="B233" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C233">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A234">
         <v>426100</v>
       </c>
-      <c r="B233" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C233">
+      <c r="B234" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C234">
         <v>80</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A234" t="s">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
         <v>64</v>
-      </c>
-      <c r="B234" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C234">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A235">
-        <v>426100</v>
       </c>
       <c r="B235" s="1" t="s">
         <v>1</v>
@@ -3453,18 +3456,18 @@
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236">
+        <v>426100</v>
+      </c>
+      <c r="B236" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C236">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A237">
         <v>416112</v>
-      </c>
-      <c r="B236" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C236">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A237" t="s">
-        <v>63</v>
       </c>
       <c r="B237" s="1" t="s">
         <v>1</v>
@@ -3475,7 +3478,7 @@
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B238" s="1" t="s">
         <v>1</v>
@@ -3486,21 +3489,21 @@
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
+        <v>65</v>
+      </c>
+      <c r="B239" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C239">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
         <v>66</v>
       </c>
-      <c r="B239" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C239">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A240">
-        <v>406115</v>
-      </c>
       <c r="B240" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C240">
         <v>80</v>
@@ -3511,21 +3514,21 @@
         <v>406115</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C241">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242">
-        <v>666001</v>
+        <v>406115</v>
       </c>
       <c r="B242" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C242">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
@@ -3533,10 +3536,10 @@
         <v>666001</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C243">
-        <v>30</v>
+        <v>120</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
@@ -3544,54 +3547,54 @@
         <v>666001</v>
       </c>
       <c r="B244" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C244">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245">
-        <v>550801</v>
+        <v>666001</v>
       </c>
       <c r="B245" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C245">
-        <v>90</v>
+        <v>40</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246">
+        <v>550801</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C246">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A247">
         <v>553424</v>
       </c>
-      <c r="B246" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C246">
+      <c r="B247" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C247">
         <v>100</v>
-      </c>
-    </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A247" t="s">
-        <v>67</v>
-      </c>
-      <c r="B247" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C247">
-        <v>150</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B248" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C248">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
@@ -3599,18 +3602,18 @@
         <v>68</v>
       </c>
       <c r="B249" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C249">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>176</v>
+        <v>68</v>
       </c>
       <c r="B250" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C250">
         <v>90</v>
@@ -3618,7 +3621,7 @@
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>69</v>
+        <v>176</v>
       </c>
       <c r="B251" s="1" t="s">
         <v>30</v>
@@ -3629,40 +3632,40 @@
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B252" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C252">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B253" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C253">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
+        <v>71</v>
+      </c>
+      <c r="B254" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C254">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A255" t="s">
         <v>72</v>
-      </c>
-      <c r="B254" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C254">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A255">
-        <v>721015</v>
       </c>
       <c r="B255" s="1" t="s">
         <v>30</v>
@@ -3673,7 +3676,7 @@
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256">
-        <v>721009</v>
+        <v>721015</v>
       </c>
       <c r="B256" s="1" t="s">
         <v>30</v>
@@ -3684,7 +3687,7 @@
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257">
-        <v>341040</v>
+        <v>721009</v>
       </c>
       <c r="B257" s="1" t="s">
         <v>30</v>
@@ -3695,7 +3698,7 @@
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258">
-        <v>341030</v>
+        <v>341040</v>
       </c>
       <c r="B258" s="1" t="s">
         <v>30</v>
@@ -3709,15 +3712,15 @@
         <v>341030</v>
       </c>
       <c r="B259" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C259">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260">
-        <v>341040</v>
+        <v>341030</v>
       </c>
       <c r="B260" s="1" t="s">
         <v>1</v>
@@ -3728,7 +3731,7 @@
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261">
-        <v>721009</v>
+        <v>341040</v>
       </c>
       <c r="B261" s="1" t="s">
         <v>1</v>
@@ -3739,7 +3742,7 @@
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262">
-        <v>721015</v>
+        <v>721009</v>
       </c>
       <c r="B262" s="1" t="s">
         <v>1</v>
@@ -3749,8 +3752,8 @@
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A263" t="s">
-        <v>72</v>
+      <c r="A263">
+        <v>721015</v>
       </c>
       <c r="B263" s="1" t="s">
         <v>1</v>
@@ -3761,7 +3764,7 @@
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B264" s="1" t="s">
         <v>1</v>
@@ -3772,46 +3775,46 @@
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B265" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C265">
-        <v>110</v>
+        <v>55</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B266" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C266">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B267" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C267">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B268" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C268">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.25">
@@ -3819,37 +3822,37 @@
         <v>74</v>
       </c>
       <c r="B269" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C269">
-        <v>75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B270" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C270">
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B271" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C271">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B272" s="1" t="s">
         <v>30</v>
@@ -3860,7 +3863,7 @@
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B273" s="1" t="s">
         <v>30</v>
@@ -3870,58 +3873,58 @@
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A274">
-        <v>720024</v>
+      <c r="A274" t="s">
+        <v>77</v>
       </c>
       <c r="B274" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C274">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275">
+        <v>720024</v>
+      </c>
+      <c r="B275" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C275">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A276">
         <v>720022</v>
       </c>
-      <c r="B275" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C275">
+      <c r="B276" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C276">
         <v>70</v>
-      </c>
-    </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A276" t="s">
-        <v>78</v>
-      </c>
-      <c r="B276" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C276">
-        <v>80</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
+        <v>78</v>
+      </c>
+      <c r="B277" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C277">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
         <v>79</v>
       </c>
-      <c r="B277" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C277">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A278">
-        <v>661000</v>
-      </c>
       <c r="B278" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C278">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.25">
@@ -3929,15 +3932,15 @@
         <v>661000</v>
       </c>
       <c r="B279" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C279">
         <v>70</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A280" t="s">
-        <v>78</v>
+      <c r="A280">
+        <v>661000</v>
       </c>
       <c r="B280" s="1" t="s">
         <v>1</v>
@@ -3948,7 +3951,7 @@
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B281" s="1" t="s">
         <v>1</v>
@@ -3958,8 +3961,8 @@
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A282">
-        <v>720022</v>
+      <c r="A282" t="s">
+        <v>79</v>
       </c>
       <c r="B282" s="1" t="s">
         <v>1</v>
@@ -3970,7 +3973,7 @@
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283">
-        <v>720024</v>
+        <v>720022</v>
       </c>
       <c r="B283" s="1" t="s">
         <v>1</v>
@@ -3980,8 +3983,8 @@
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A284" t="s">
-        <v>77</v>
+      <c r="A284">
+        <v>720024</v>
       </c>
       <c r="B284" s="1" t="s">
         <v>1</v>
@@ -3992,46 +3995,46 @@
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B285" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C285">
-        <v>110</v>
+        <v>70</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B286" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C286">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
+        <v>75</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C287">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
         <v>80</v>
       </c>
-      <c r="B287" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C287">
+      <c r="B288" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C288">
         <v>100</v>
-      </c>
-    </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A288">
-        <v>416210</v>
-      </c>
-      <c r="B288" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C288">
-        <v>0</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
@@ -4039,54 +4042,54 @@
         <v>416210</v>
       </c>
       <c r="B289" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C289">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A290">
+        <v>416210</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C290">
         <v>100</v>
       </c>
     </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A290" t="s">
+    <row r="291" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A291" t="s">
         <v>80</v>
       </c>
-      <c r="B290" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C290">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A291">
-        <v>406210</v>
-      </c>
       <c r="B291" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C291">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A292">
-        <v>650050</v>
+        <v>406210</v>
       </c>
       <c r="B292" s="1" t="s">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="C292">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A293">
-        <v>650040</v>
+        <v>650050</v>
       </c>
       <c r="B293" s="1" t="s">
         <v>81</v>
       </c>
       <c r="C293">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="294" spans="1:3" x14ac:dyDescent="0.25">
@@ -4094,10 +4097,10 @@
         <v>650040</v>
       </c>
       <c r="B294" s="1" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="C294">
-        <v>140</v>
+        <v>90</v>
       </c>
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
@@ -4105,21 +4108,21 @@
         <v>650040</v>
       </c>
       <c r="B295" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C295">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="296" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A296">
-        <v>650050</v>
+        <v>650040</v>
       </c>
       <c r="B296" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C296">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.25">
@@ -4127,21 +4130,21 @@
         <v>650050</v>
       </c>
       <c r="B297" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C297">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298">
-        <v>650020</v>
+        <v>650050</v>
       </c>
       <c r="B298" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C298">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="299" spans="1:3" x14ac:dyDescent="0.25">
@@ -4149,21 +4152,21 @@
         <v>650020</v>
       </c>
       <c r="B299" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C299">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="300" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A300">
-        <v>600138</v>
+        <v>650020</v>
       </c>
       <c r="B300" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C300">
-        <v>170</v>
+        <v>100</v>
       </c>
     </row>
     <row r="301" spans="1:3" x14ac:dyDescent="0.25">
@@ -4171,26 +4174,26 @@
         <v>600138</v>
       </c>
       <c r="B301" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C301">
-        <v>150</v>
+        <v>170</v>
       </c>
     </row>
     <row r="302" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A302">
-        <v>600121</v>
+        <v>600138</v>
       </c>
       <c r="B302" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C302">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="303" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A303">
-        <v>600127</v>
+        <v>600121</v>
       </c>
       <c r="B303" s="1" t="s">
         <v>30</v>
@@ -4201,7 +4204,7 @@
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A304">
-        <v>600227</v>
+        <v>600127</v>
       </c>
       <c r="B304" s="1" t="s">
         <v>30</v>
@@ -4215,26 +4218,26 @@
         <v>600227</v>
       </c>
       <c r="B305" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C305">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A306">
-        <v>600127</v>
+        <v>600227</v>
       </c>
       <c r="B306" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C306">
-        <v>90</v>
+        <v>150</v>
       </c>
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307">
-        <v>600121</v>
+        <v>600127</v>
       </c>
       <c r="B307" s="1" t="s">
         <v>1</v>
@@ -4245,13 +4248,13 @@
     </row>
     <row r="308" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A308">
-        <v>600128</v>
+        <v>600121</v>
       </c>
       <c r="B308" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C308">
-        <v>150</v>
+        <v>90</v>
       </c>
     </row>
     <row r="309" spans="1:3" x14ac:dyDescent="0.25">
@@ -4259,21 +4262,21 @@
         <v>600128</v>
       </c>
       <c r="B309" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C309">
-        <v>70</v>
+        <v>150</v>
       </c>
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A310">
-        <v>650030</v>
+        <v>600128</v>
       </c>
       <c r="B310" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C310">
-        <v>170</v>
+        <v>70</v>
       </c>
     </row>
     <row r="311" spans="1:3" x14ac:dyDescent="0.25">
@@ -4281,21 +4284,21 @@
         <v>650030</v>
       </c>
       <c r="B311" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C311">
-        <v>70</v>
+        <v>170</v>
       </c>
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A312">
-        <v>660000</v>
+        <v>650030</v>
       </c>
       <c r="B312" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C312">
-        <v>120</v>
+        <v>70</v>
       </c>
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.25">
@@ -4303,21 +4306,21 @@
         <v>660000</v>
       </c>
       <c r="B313" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C313">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A314">
+        <v>660000</v>
+      </c>
+      <c r="B314" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C314">
         <v>80</v>
-      </c>
-    </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A314" t="s">
-        <v>82</v>
-      </c>
-      <c r="B314" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C314">
-        <v>110</v>
       </c>
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.25">
@@ -4325,18 +4328,18 @@
         <v>82</v>
       </c>
       <c r="B315" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C315">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B316" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C316">
         <v>0</v>
@@ -4347,7 +4350,7 @@
         <v>83</v>
       </c>
       <c r="B317" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C317">
         <v>0</v>
@@ -4358,32 +4361,32 @@
         <v>83</v>
       </c>
       <c r="B318" s="1" t="s">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="C318">
-        <v>120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B319" s="1" t="s">
         <v>81</v>
       </c>
       <c r="C319">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="320" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A320">
-        <v>406670</v>
+      <c r="A320" t="s">
+        <v>82</v>
       </c>
       <c r="B320" s="1" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="C320">
-        <v>110</v>
+        <v>0</v>
       </c>
     </row>
     <row r="321" spans="1:3" x14ac:dyDescent="0.25">
@@ -4391,32 +4394,32 @@
         <v>406670</v>
       </c>
       <c r="B321" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C321">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322">
+        <v>406670</v>
+      </c>
+      <c r="B322" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C322">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A323">
         <v>406316</v>
       </c>
-      <c r="B322" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C322">
+      <c r="B323" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C323">
         <v>120</v>
-      </c>
-    </row>
-    <row r="323" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A323" t="s">
-        <v>84</v>
-      </c>
-      <c r="B323" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C323">
-        <v>80</v>
       </c>
     </row>
     <row r="324" spans="1:3" x14ac:dyDescent="0.25">
@@ -4424,21 +4427,21 @@
         <v>84</v>
       </c>
       <c r="B324" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C324">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="325" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B325" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C325">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.25">
@@ -4446,59 +4449,59 @@
         <v>85</v>
       </c>
       <c r="B326" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C326">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="327" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
+        <v>85</v>
+      </c>
+      <c r="B327" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C327">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A328" t="s">
         <v>86</v>
       </c>
-      <c r="B327" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C327">
+      <c r="B328" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C328">
         <v>60</v>
       </c>
     </row>
-    <row r="328" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A328">
+    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A329">
         <v>550800</v>
       </c>
-      <c r="B328" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C328">
+      <c r="B329" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C329">
         <v>80</v>
-      </c>
-    </row>
-    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A329" t="s">
-        <v>87</v>
-      </c>
-      <c r="B329" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C329">
-        <v>90</v>
       </c>
     </row>
     <row r="330" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B330" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C330">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="331" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B331" s="1" t="s">
         <v>30</v>
@@ -4509,18 +4512,18 @@
     </row>
     <row r="332" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B332" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C332">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="333" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B333" s="1" t="s">
         <v>30</v>
@@ -4531,73 +4534,73 @@
     </row>
     <row r="334" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B334" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C334">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="335" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
+        <v>92</v>
+      </c>
+      <c r="B335" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C335">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="336" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A336" t="s">
         <v>93</v>
       </c>
-      <c r="B335" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C335">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="336" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A336">
+      <c r="B336" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C336">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="337" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A337">
         <v>720023</v>
       </c>
-      <c r="B336" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C336">
+      <c r="B337" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C337">
         <v>80</v>
       </c>
     </row>
-    <row r="337" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A337" t="s">
+    <row r="338" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A338" t="s">
         <v>94</v>
       </c>
-      <c r="B337" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C337">
+      <c r="B338" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C338">
         <v>70</v>
-      </c>
-    </row>
-    <row r="338" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A338">
-        <v>240040</v>
-      </c>
-      <c r="B338" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C338">
-        <v>60</v>
       </c>
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A339">
-        <v>240030</v>
+        <v>240040</v>
       </c>
       <c r="B339" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C339">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A340">
-        <v>240020</v>
+        <v>240030</v>
       </c>
       <c r="B340" s="1" t="s">
         <v>30</v>
@@ -4611,26 +4614,26 @@
         <v>240020</v>
       </c>
       <c r="B341" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C341">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="342" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A342">
-        <v>240030</v>
+        <v>240020</v>
       </c>
       <c r="B342" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C342">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="343" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A343">
-        <v>240040</v>
+        <v>240030</v>
       </c>
       <c r="B343" s="1" t="s">
         <v>1</v>
@@ -4640,8 +4643,8 @@
       </c>
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A344" t="s">
-        <v>94</v>
+      <c r="A344">
+        <v>240040</v>
       </c>
       <c r="B344" s="1" t="s">
         <v>1</v>
@@ -4651,19 +4654,19 @@
       </c>
     </row>
     <row r="345" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A345">
+      <c r="A345" t="s">
+        <v>94</v>
+      </c>
+      <c r="B345" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C345">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A346">
         <v>720023</v>
-      </c>
-      <c r="B345" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C345">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="346" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A346" t="s">
-        <v>93</v>
       </c>
       <c r="B346" s="1" t="s">
         <v>1</v>
@@ -4674,40 +4677,40 @@
     </row>
     <row r="347" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B347" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C347">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="348" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B348" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C348">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="349" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B349" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C349">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="350" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B350" s="1" t="s">
         <v>1</v>
@@ -4718,18 +4721,18 @@
     </row>
     <row r="351" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B351" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C351">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="352" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B352" s="1" t="s">
         <v>1</v>
@@ -4740,35 +4743,35 @@
     </row>
     <row r="353" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C353">
-        <v>80</v>
+        <v>50</v>
       </c>
     </row>
     <row r="354" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B354" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C354">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="355" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B355" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C355">
-        <v>45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="356" spans="1:3" x14ac:dyDescent="0.25">
@@ -4776,15 +4779,15 @@
         <v>97</v>
       </c>
       <c r="B356" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C356">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="357" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B357" s="1" t="s">
         <v>1</v>
@@ -4795,40 +4798,40 @@
     </row>
     <row r="358" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
+        <v>96</v>
+      </c>
+      <c r="B358" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C358">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="359" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A359" t="s">
         <v>95</v>
       </c>
-      <c r="B358" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C358">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="359" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A359">
-        <v>722010</v>
-      </c>
       <c r="B359" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C359">
-        <v>80</v>
+        <v>30</v>
       </c>
     </row>
     <row r="360" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A360">
-        <v>722005</v>
+        <v>722010</v>
       </c>
       <c r="B360" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C360">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="361" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A361">
-        <v>722006</v>
+        <v>722005</v>
       </c>
       <c r="B361" s="1" t="s">
         <v>30</v>
@@ -4839,13 +4842,13 @@
     </row>
     <row r="362" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A362">
-        <v>722000</v>
+        <v>722006</v>
       </c>
       <c r="B362" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C362">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="363" spans="1:3" x14ac:dyDescent="0.25">
@@ -4853,7 +4856,7 @@
         <v>722000</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C363">
         <v>60</v>
@@ -4861,18 +4864,18 @@
     </row>
     <row r="364" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A364">
-        <v>722006</v>
+        <v>722000</v>
       </c>
       <c r="B364" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C364">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="365" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A365">
-        <v>722005</v>
+        <v>722006</v>
       </c>
       <c r="B365" s="1" t="s">
         <v>1</v>
@@ -4883,40 +4886,40 @@
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A366">
+        <v>722005</v>
+      </c>
+      <c r="B366" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C366">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A367">
         <v>722010</v>
       </c>
-      <c r="B366" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C366">
+      <c r="B367" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C367">
         <v>50</v>
-      </c>
-    </row>
-    <row r="367" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A367" t="s">
-        <v>98</v>
-      </c>
-      <c r="B367" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C367">
-        <v>80</v>
       </c>
     </row>
     <row r="368" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B368" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C368">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="369" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B369" s="1" t="s">
         <v>30</v>
@@ -4927,13 +4930,13 @@
     </row>
     <row r="370" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B370" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C370">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="371" spans="1:3" x14ac:dyDescent="0.25">
@@ -4941,7 +4944,7 @@
         <v>101</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C371">
         <v>60</v>
@@ -4949,29 +4952,29 @@
     </row>
     <row r="372" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B372" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C372">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="373" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B373" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C373">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="374" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B374" s="1" t="s">
         <v>1</v>
@@ -4982,40 +4985,40 @@
     </row>
     <row r="375" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B375" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C375">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="376" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B376" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C376">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="377" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B377" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C377">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="378" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B378" s="1" t="s">
         <v>30</v>
@@ -5029,26 +5032,26 @@
         <v>105</v>
       </c>
       <c r="B379" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C379">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="380" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B380" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C380">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="381" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B381" s="1" t="s">
         <v>1</v>
@@ -5059,35 +5062,35 @@
     </row>
     <row r="382" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B382" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C382">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="383" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B383" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C383">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="384" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B384" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C384">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="385" spans="1:3" x14ac:dyDescent="0.25">
@@ -5095,70 +5098,70 @@
         <v>107</v>
       </c>
       <c r="B385" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C385">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="386" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
+        <v>107</v>
+      </c>
+      <c r="B386" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C386">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="387" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A387" t="s">
         <v>106</v>
       </c>
-      <c r="B386" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C386">
+      <c r="B387" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C387">
         <v>60</v>
-      </c>
-    </row>
-    <row r="387" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A387">
-        <v>406010</v>
-      </c>
-      <c r="B387" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C387">
-        <v>120</v>
       </c>
     </row>
     <row r="388" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A388">
-        <v>406321</v>
+        <v>406010</v>
       </c>
       <c r="B388" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C388">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="389" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A389">
-        <v>406660</v>
+        <v>406321</v>
       </c>
       <c r="B389" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C389">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="390" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A390">
-        <v>406329</v>
+        <v>406660</v>
       </c>
       <c r="B390" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C390">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="391" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A391">
-        <v>406325</v>
+        <v>406329</v>
       </c>
       <c r="B391" s="1" t="s">
         <v>1</v>
@@ -5169,13 +5172,13 @@
     </row>
     <row r="392" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A392">
-        <v>416240</v>
+        <v>406325</v>
       </c>
       <c r="B392" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C392">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="393" spans="1:3" x14ac:dyDescent="0.25">
@@ -5183,15 +5186,15 @@
         <v>416240</v>
       </c>
       <c r="B393" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C393">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="394" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A394" t="s">
-        <v>108</v>
+      <c r="A394">
+        <v>416240</v>
       </c>
       <c r="B394" s="1" t="s">
         <v>1</v>
@@ -5202,10 +5205,10 @@
     </row>
     <row r="395" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B395" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C395">
         <v>100</v>
@@ -5216,21 +5219,21 @@
         <v>109</v>
       </c>
       <c r="B396" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C396">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="397" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B397" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C397">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="398" spans="1:3" x14ac:dyDescent="0.25">
@@ -5238,7 +5241,7 @@
         <v>110</v>
       </c>
       <c r="B398" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C398">
         <v>100</v>
@@ -5246,10 +5249,10 @@
     </row>
     <row r="399" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B399" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C399">
         <v>100</v>
@@ -5260,18 +5263,18 @@
         <v>111</v>
       </c>
       <c r="B400" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C400">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="401" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B401" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C401">
         <v>90</v>
@@ -5282,21 +5285,21 @@
         <v>112</v>
       </c>
       <c r="B402" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C402">
-        <v>130</v>
+        <v>90</v>
       </c>
     </row>
     <row r="403" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B403" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C403">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="404" spans="1:3" x14ac:dyDescent="0.25">
@@ -5304,21 +5307,21 @@
         <v>113</v>
       </c>
       <c r="B404" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C404">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="405" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A405" t="s">
+        <v>113</v>
+      </c>
+      <c r="B405" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C405">
         <v>130</v>
-      </c>
-    </row>
-    <row r="405" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A405">
-        <v>242320</v>
-      </c>
-      <c r="B405" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C405">
-        <v>100</v>
       </c>
     </row>
     <row r="406" spans="1:3" x14ac:dyDescent="0.25">
@@ -5326,7 +5329,7 @@
         <v>242320</v>
       </c>
       <c r="B406" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C406">
         <v>100</v>
@@ -5334,13 +5337,13 @@
     </row>
     <row r="407" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A407">
-        <v>651050</v>
+        <v>242320</v>
       </c>
       <c r="B407" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C407">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="408" spans="1:3" x14ac:dyDescent="0.25">
@@ -5348,7 +5351,7 @@
         <v>651050</v>
       </c>
       <c r="B408" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C408">
         <v>110</v>
@@ -5356,13 +5359,13 @@
     </row>
     <row r="409" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A409">
-        <v>730010</v>
+        <v>651050</v>
       </c>
       <c r="B409" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C409">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="410" spans="1:3" x14ac:dyDescent="0.25">
@@ -5370,7 +5373,7 @@
         <v>730010</v>
       </c>
       <c r="B410" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C410">
         <v>100</v>
@@ -5378,10 +5381,10 @@
     </row>
     <row r="411" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A411">
-        <v>731020</v>
+        <v>730010</v>
       </c>
       <c r="B411" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C411">
         <v>100</v>
@@ -5392,21 +5395,21 @@
         <v>731020</v>
       </c>
       <c r="B412" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C412">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="413" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A413">
-        <v>476273</v>
+        <v>731020</v>
       </c>
       <c r="B413" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C413">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="414" spans="1:3" x14ac:dyDescent="0.25">
@@ -5414,21 +5417,21 @@
         <v>476273</v>
       </c>
       <c r="B414" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C414">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="415" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A415" t="s">
-        <v>114</v>
+      <c r="A415">
+        <v>476273</v>
       </c>
       <c r="B415" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C415">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="416" spans="1:3" x14ac:dyDescent="0.25">
@@ -5436,21 +5439,21 @@
         <v>114</v>
       </c>
       <c r="B416" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C416">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="417" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A417">
-        <v>466009</v>
+      <c r="A417" t="s">
+        <v>114</v>
       </c>
       <c r="B417" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C417">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="418" spans="1:3" x14ac:dyDescent="0.25">
@@ -5458,21 +5461,21 @@
         <v>466009</v>
       </c>
       <c r="B418" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C418">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="419" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A419">
-        <v>416273</v>
+        <v>466009</v>
       </c>
       <c r="B419" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C419">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="420" spans="1:3" x14ac:dyDescent="0.25">
@@ -5480,21 +5483,21 @@
         <v>416273</v>
       </c>
       <c r="B420" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C420">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="421" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A421">
-        <v>466023</v>
+        <v>416273</v>
       </c>
       <c r="B421" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C421">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="422" spans="1:3" x14ac:dyDescent="0.25">
@@ -5502,21 +5505,21 @@
         <v>466023</v>
       </c>
       <c r="B422" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C422">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="423" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A423">
-        <v>426200</v>
+        <v>466023</v>
       </c>
       <c r="B423" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C423">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="424" spans="1:3" x14ac:dyDescent="0.25">
@@ -5524,21 +5527,21 @@
         <v>426200</v>
       </c>
       <c r="B424" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C424">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="425" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A425">
-        <v>406272</v>
+        <v>426200</v>
       </c>
       <c r="B425" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C425">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="426" spans="1:3" x14ac:dyDescent="0.25">
@@ -5546,21 +5549,21 @@
         <v>406272</v>
       </c>
       <c r="B426" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C426">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="427" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A427" t="s">
-        <v>115</v>
+      <c r="A427">
+        <v>406272</v>
       </c>
       <c r="B427" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C427">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="428" spans="1:3" x14ac:dyDescent="0.25">
@@ -5568,18 +5571,18 @@
         <v>115</v>
       </c>
       <c r="B428" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C428">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="429" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B429" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C429">
         <v>80</v>
@@ -5590,7 +5593,7 @@
         <v>116</v>
       </c>
       <c r="B430" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C430">
         <v>80</v>
@@ -5598,10 +5601,10 @@
     </row>
     <row r="431" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B431" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C431">
         <v>80</v>
@@ -5612,147 +5615,147 @@
         <v>117</v>
       </c>
       <c r="B432" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C432">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="433" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A433">
-        <v>416338</v>
+      <c r="A433" t="s">
+        <v>117</v>
       </c>
       <c r="B433" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C433">
-        <v>150</v>
+        <v>0</v>
       </c>
     </row>
     <row r="434" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A434">
-        <v>416331</v>
+        <v>416338</v>
       </c>
       <c r="B434" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C434">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="435" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A435">
-        <v>416065</v>
+        <v>416331</v>
       </c>
       <c r="B435" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C435">
-        <v>90</v>
+        <v>200</v>
       </c>
     </row>
     <row r="436" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A436">
-        <v>416067</v>
+        <v>416065</v>
       </c>
       <c r="B436" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C436">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="437" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A437">
-        <v>416086</v>
+        <v>416067</v>
       </c>
       <c r="B437" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C437">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="438" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A438">
+        <v>416086</v>
+      </c>
+      <c r="B438" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C438">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="439" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A439">
         <v>416096</v>
       </c>
-      <c r="B438" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C438">
+      <c r="B439" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C439">
         <v>120</v>
       </c>
     </row>
-    <row r="439" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A439" t="s">
+    <row r="440" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A440" t="s">
         <v>118</v>
       </c>
-      <c r="B439" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C439">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="440" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A440">
-        <v>666003</v>
-      </c>
       <c r="B440" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C440">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="441" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A441">
+        <v>666003</v>
+      </c>
+      <c r="B441" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C441">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="442" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A442">
         <v>666002</v>
       </c>
-      <c r="B441" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C441">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="442" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A442" t="s">
+      <c r="B442" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C442">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="443" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A443" t="s">
         <v>119</v>
       </c>
-      <c r="B442" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C442">
+      <c r="B443" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C443">
         <v>85</v>
-      </c>
-    </row>
-    <row r="443" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A443">
-        <v>416070</v>
-      </c>
-      <c r="B443" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C443">
-        <v>90</v>
       </c>
     </row>
     <row r="444" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A444">
+        <v>416070</v>
+      </c>
+      <c r="B444" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C444">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="445" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A445">
         <v>416069</v>
-      </c>
-      <c r="B444" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C444">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="445" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A445" t="s">
-        <v>120</v>
       </c>
       <c r="B445" s="1" t="s">
         <v>1</v>
@@ -5762,8 +5765,8 @@
       </c>
     </row>
     <row r="446" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A446">
-        <v>406340</v>
+      <c r="A446" t="s">
+        <v>120</v>
       </c>
       <c r="B446" s="1" t="s">
         <v>1</v>
@@ -5774,7 +5777,7 @@
     </row>
     <row r="447" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A447">
-        <v>416301</v>
+        <v>406340</v>
       </c>
       <c r="B447" s="1" t="s">
         <v>1</v>
@@ -5785,35 +5788,35 @@
     </row>
     <row r="448" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A448">
-        <v>416119</v>
+        <v>416301</v>
       </c>
       <c r="B448" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C448">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="449" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A449">
-        <v>406081</v>
+        <v>416119</v>
       </c>
       <c r="B449" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C449">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="450" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A450">
-        <v>416068</v>
+        <v>406081</v>
       </c>
       <c r="B450" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C450">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="451" spans="1:3" x14ac:dyDescent="0.25">
@@ -5821,48 +5824,48 @@
         <v>416068</v>
       </c>
       <c r="B451" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C451">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="452" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A452">
-        <v>736315</v>
+        <v>416068</v>
       </c>
       <c r="B452" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C452">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="453" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A453">
+        <v>736315</v>
+      </c>
+      <c r="B453" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C453">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="454" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A454">
         <v>736334</v>
       </c>
-      <c r="B453" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C453">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="454" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A454" t="s">
+      <c r="B454" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C454">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="455" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A455" t="s">
         <v>121</v>
-      </c>
-      <c r="B454" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C454">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="455" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A455">
-        <v>406307</v>
       </c>
       <c r="B455" s="1" t="s">
         <v>1</v>
@@ -5873,7 +5876,7 @@
     </row>
     <row r="456" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A456">
-        <v>466400</v>
+        <v>406307</v>
       </c>
       <c r="B456" s="1" t="s">
         <v>1</v>
@@ -5884,13 +5887,13 @@
     </row>
     <row r="457" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A457">
-        <v>416139</v>
+        <v>466400</v>
       </c>
       <c r="B457" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C457">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="458" spans="1:3" x14ac:dyDescent="0.25">
@@ -5898,7 +5901,7 @@
         <v>416139</v>
       </c>
       <c r="B458" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C458">
         <v>80</v>
@@ -5906,7 +5909,7 @@
     </row>
     <row r="459" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A459">
-        <v>416148</v>
+        <v>416139</v>
       </c>
       <c r="B459" s="1" t="s">
         <v>1</v>
@@ -5916,30 +5919,30 @@
       </c>
     </row>
     <row r="460" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A460" t="s">
-        <v>122</v>
+      <c r="A460">
+        <v>416148</v>
       </c>
       <c r="B460" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C460">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="461" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B461" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C461">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="462" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B462" s="1" t="s">
         <v>1</v>
@@ -5950,7 +5953,7 @@
     </row>
     <row r="463" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B463" s="1" t="s">
         <v>1</v>
@@ -5961,40 +5964,40 @@
     </row>
     <row r="464" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B464" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C464">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="465" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B465" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C465">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="466" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B466" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C466">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="467" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>171</v>
+        <v>128</v>
       </c>
       <c r="B467" s="1" t="s">
         <v>1</v>
@@ -6004,30 +6007,30 @@
       </c>
     </row>
     <row r="468" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A468">
+      <c r="A468" t="s">
+        <v>171</v>
+      </c>
+      <c r="B468" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C468">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="469" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A469">
         <v>406310</v>
       </c>
-      <c r="B468" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C468">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="469" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A469" t="s">
+      <c r="B469" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C469">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="470" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A470" t="s">
         <v>129</v>
-      </c>
-      <c r="B469" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C469">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="470" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A470">
-        <v>416180</v>
       </c>
       <c r="B470" s="1" t="s">
         <v>1</v>
@@ -6038,7 +6041,7 @@
     </row>
     <row r="471" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A471">
-        <v>606180</v>
+        <v>416180</v>
       </c>
       <c r="B471" s="1" t="s">
         <v>1</v>
@@ -6049,7 +6052,7 @@
     </row>
     <row r="472" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A472">
-        <v>656310</v>
+        <v>606180</v>
       </c>
       <c r="B472" s="1" t="s">
         <v>1</v>
@@ -6060,7 +6063,7 @@
     </row>
     <row r="473" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A473">
-        <v>416311</v>
+        <v>656310</v>
       </c>
       <c r="B473" s="1" t="s">
         <v>1</v>
@@ -6071,7 +6074,7 @@
     </row>
     <row r="474" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A474">
-        <v>406157</v>
+        <v>416311</v>
       </c>
       <c r="B474" s="1" t="s">
         <v>1</v>
@@ -6082,7 +6085,7 @@
     </row>
     <row r="475" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A475">
-        <v>416182</v>
+        <v>406157</v>
       </c>
       <c r="B475" s="1" t="s">
         <v>1</v>
@@ -6093,18 +6096,18 @@
     </row>
     <row r="476" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A476">
-        <v>406315</v>
+        <v>416182</v>
       </c>
       <c r="B476" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C476">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="477" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A477">
-        <v>406312</v>
+        <v>406315</v>
       </c>
       <c r="B477" s="1" t="s">
         <v>1</v>
@@ -6114,19 +6117,19 @@
       </c>
     </row>
     <row r="478" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A478" t="s">
-        <v>130</v>
+      <c r="A478">
+        <v>406312</v>
       </c>
       <c r="B478" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C478">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="479" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B479" s="1" t="s">
         <v>30</v>
@@ -6140,15 +6143,15 @@
         <v>131</v>
       </c>
       <c r="B480" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C480">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="481" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B481" s="1" t="s">
         <v>1</v>
@@ -6158,14 +6161,14 @@
       </c>
     </row>
     <row r="482" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A482">
-        <v>762013</v>
+      <c r="A482" t="s">
+        <v>130</v>
       </c>
       <c r="B482" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C482">
-        <v>85</v>
+        <v>70</v>
       </c>
     </row>
     <row r="483" spans="1:3" x14ac:dyDescent="0.25">
@@ -6173,21 +6176,21 @@
         <v>762013</v>
       </c>
       <c r="B483" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C483">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="484" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A484">
+        <v>762013</v>
+      </c>
+      <c r="B484" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C484">
         <v>60</v>
-      </c>
-    </row>
-    <row r="484" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A484" t="s">
-        <v>132</v>
-      </c>
-      <c r="B484" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C484">
-        <v>90</v>
       </c>
     </row>
     <row r="485" spans="1:3" x14ac:dyDescent="0.25">
@@ -6195,21 +6198,21 @@
         <v>132</v>
       </c>
       <c r="B485" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C485">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="486" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B486" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C486">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="487" spans="1:3" x14ac:dyDescent="0.25">
@@ -6217,21 +6220,21 @@
         <v>133</v>
       </c>
       <c r="B487" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C487">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="488" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B488" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C488">
-        <v>100</v>
+        <v>60</v>
       </c>
     </row>
     <row r="489" spans="1:3" x14ac:dyDescent="0.25">
@@ -6239,21 +6242,21 @@
         <v>134</v>
       </c>
       <c r="B489" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C489">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="490" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A490" t="s">
+        <v>134</v>
+      </c>
+      <c r="B490" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C490">
         <v>60</v>
-      </c>
-    </row>
-    <row r="490" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A490">
-        <v>242020</v>
-      </c>
-      <c r="B490" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C490">
-        <v>70</v>
       </c>
     </row>
     <row r="491" spans="1:3" x14ac:dyDescent="0.25">
@@ -6261,21 +6264,21 @@
         <v>242020</v>
       </c>
       <c r="B491" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C491">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="492" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A492">
-        <v>602010</v>
+        <v>242020</v>
       </c>
       <c r="B492" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C492">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="493" spans="1:3" x14ac:dyDescent="0.25">
@@ -6283,21 +6286,21 @@
         <v>602010</v>
       </c>
       <c r="B493" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C493">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="494" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A494">
-        <v>652010</v>
+        <v>602010</v>
       </c>
       <c r="B494" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C494">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="495" spans="1:3" x14ac:dyDescent="0.25">
@@ -6305,37 +6308,37 @@
         <v>652010</v>
       </c>
       <c r="B495" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C495">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="496" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A496">
+        <v>652010</v>
+      </c>
+      <c r="B496" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C496">
         <v>60</v>
-      </c>
-    </row>
-    <row r="496" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A496" t="s">
-        <v>135</v>
-      </c>
-      <c r="B496" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C496">
-        <v>70</v>
       </c>
     </row>
     <row r="497" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A497" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B497" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C497">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="498" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A498" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B498" s="1" t="s">
         <v>1</v>
@@ -6346,7 +6349,7 @@
     </row>
     <row r="499" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A499" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B499" s="1" t="s">
         <v>1</v>
@@ -6357,29 +6360,29 @@
     </row>
     <row r="500" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A500" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B500" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C500">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="501" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A501" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B501" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C501">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="502" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A502" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B502" s="1" t="s">
         <v>56</v>
@@ -6390,7 +6393,7 @@
     </row>
     <row r="503" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A503" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B503" s="1" t="s">
         <v>56</v>
@@ -6404,26 +6407,26 @@
         <v>138</v>
       </c>
       <c r="B504" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C504">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="505" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A505" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B505" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C505">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="506" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A506" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B506" s="1" t="s">
         <v>30</v>
@@ -6434,7 +6437,7 @@
     </row>
     <row r="507" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A507" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B507" s="1" t="s">
         <v>30</v>
@@ -6445,29 +6448,29 @@
     </row>
     <row r="508" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A508" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B508" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C508">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="509" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A509" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B509" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C509">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="510" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A510" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B510" s="1" t="s">
         <v>1</v>
@@ -6478,29 +6481,29 @@
     </row>
     <row r="511" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A511" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B511" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C511">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="512" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A512" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B512" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C512">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="513" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A513" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B513" s="1" t="s">
         <v>56</v>
@@ -6514,26 +6517,26 @@
         <v>141</v>
       </c>
       <c r="B514" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C514">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="515" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A515" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B515" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C515">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="516" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A516" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B516" s="1" t="s">
         <v>30</v>
@@ -6544,13 +6547,13 @@
     </row>
     <row r="517" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A517" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B517" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C517">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="518" spans="1:3" x14ac:dyDescent="0.25">
@@ -6558,10 +6561,10 @@
         <v>142</v>
       </c>
       <c r="B518" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C518">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="519" spans="1:3" x14ac:dyDescent="0.25">
@@ -6569,18 +6572,18 @@
         <v>142</v>
       </c>
       <c r="B519" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C519">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="520" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A520">
-        <v>720004</v>
+      <c r="A520" t="s">
+        <v>142</v>
       </c>
       <c r="B520" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C520">
         <v>70</v>
@@ -6588,21 +6591,21 @@
     </row>
     <row r="521" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A521">
-        <v>720003</v>
+        <v>720004</v>
       </c>
       <c r="B521" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C521">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="522" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A522">
-        <v>720004</v>
+        <v>720003</v>
       </c>
       <c r="B522" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C522">
         <v>0</v>
@@ -6610,7 +6613,7 @@
     </row>
     <row r="523" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A523">
-        <v>720003</v>
+        <v>720004</v>
       </c>
       <c r="B523" s="1" t="s">
         <v>30</v>
@@ -6624,7 +6627,7 @@
         <v>720003</v>
       </c>
       <c r="B524" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C524">
         <v>0</v>
@@ -6632,7 +6635,7 @@
     </row>
     <row r="525" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A525">
-        <v>720004</v>
+        <v>720003</v>
       </c>
       <c r="B525" s="1" t="s">
         <v>1</v>
@@ -6643,13 +6646,13 @@
     </row>
     <row r="526" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A526">
-        <v>721001</v>
+        <v>720004</v>
       </c>
       <c r="B526" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C526">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="527" spans="1:3" x14ac:dyDescent="0.25">
@@ -6657,10 +6660,10 @@
         <v>721001</v>
       </c>
       <c r="B527" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C527">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="528" spans="1:3" x14ac:dyDescent="0.25">
@@ -6668,7 +6671,7 @@
         <v>721001</v>
       </c>
       <c r="B528" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C528">
         <v>0</v>
@@ -6676,13 +6679,13 @@
     </row>
     <row r="529" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A529">
-        <v>651030</v>
+        <v>721001</v>
       </c>
       <c r="B529" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C529">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="530" spans="1:3" x14ac:dyDescent="0.25">
@@ -6690,21 +6693,21 @@
         <v>651030</v>
       </c>
       <c r="B530" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C530">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="531" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A531">
-        <v>651010</v>
+        <v>651030</v>
       </c>
       <c r="B531" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C531">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="532" spans="1:3" x14ac:dyDescent="0.25">
@@ -6712,37 +6715,37 @@
         <v>651010</v>
       </c>
       <c r="B532" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C532">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="533" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A533" t="s">
-        <v>143</v>
+      <c r="A533">
+        <v>651010</v>
       </c>
       <c r="B533" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C533">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="534" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A534" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B534" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C534">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="535" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A535" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B535" s="1" t="s">
         <v>1</v>
@@ -6753,7 +6756,7 @@
     </row>
     <row r="536" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A536" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B536" s="1" t="s">
         <v>1</v>
@@ -6764,10 +6767,10 @@
     </row>
     <row r="537" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A537" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B537" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C537">
         <v>0</v>
@@ -6775,7 +6778,7 @@
     </row>
     <row r="538" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A538" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B538" s="1" t="s">
         <v>56</v>
@@ -6786,7 +6789,7 @@
     </row>
     <row r="539" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A539" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B539" s="1" t="s">
         <v>56</v>
@@ -6797,7 +6800,7 @@
     </row>
     <row r="540" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A540" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B540" s="1" t="s">
         <v>56</v>
@@ -6808,10 +6811,10 @@
     </row>
     <row r="541" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A541" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B541" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C541">
         <v>0</v>
@@ -6819,7 +6822,7 @@
     </row>
     <row r="542" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A542" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B542" s="1" t="s">
         <v>30</v>
@@ -6830,7 +6833,7 @@
     </row>
     <row r="543" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A543" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B543" s="1" t="s">
         <v>30</v>
@@ -6841,7 +6844,7 @@
     </row>
     <row r="544" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A544" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B544" s="1" t="s">
         <v>30</v>
@@ -6852,32 +6855,32 @@
     </row>
     <row r="545" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A545" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B545" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C545">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="546" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A546" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B546" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C546">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="547" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A547" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B547" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C547">
         <v>0</v>
@@ -6885,7 +6888,7 @@
     </row>
     <row r="548" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A548" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B548" s="1" t="s">
         <v>56</v>
@@ -6896,10 +6899,10 @@
     </row>
     <row r="549" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A549" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B549" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C549">
         <v>0</v>
@@ -6907,7 +6910,7 @@
     </row>
     <row r="550" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A550" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B550" s="1" t="s">
         <v>30</v>
@@ -6918,13 +6921,13 @@
     </row>
     <row r="551" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A551" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B551" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C551">
-        <v>110</v>
+        <v>0</v>
       </c>
     </row>
     <row r="552" spans="1:3" x14ac:dyDescent="0.25">
@@ -6932,15 +6935,15 @@
         <v>149</v>
       </c>
       <c r="B552" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C552">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="553" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A553" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B553" s="1" t="s">
         <v>30</v>
@@ -6954,32 +6957,32 @@
         <v>150</v>
       </c>
       <c r="B554" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C554">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="555" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A555" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B555" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C555">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="556" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A556" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B556" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C556">
-        <v>150</v>
+        <v>60</v>
       </c>
     </row>
     <row r="557" spans="1:3" x14ac:dyDescent="0.25">
@@ -6987,18 +6990,18 @@
         <v>151</v>
       </c>
       <c r="B557" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C557">
-        <v>110</v>
+        <v>150</v>
       </c>
     </row>
     <row r="558" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A558">
-        <v>721014</v>
+      <c r="A558" t="s">
+        <v>151</v>
       </c>
       <c r="B558" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C558">
         <v>110</v>
@@ -7006,24 +7009,24 @@
     </row>
     <row r="559" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A559">
-        <v>721008</v>
+        <v>721014</v>
       </c>
       <c r="B559" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C559">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="560" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A560">
-        <v>721005</v>
+        <v>721008</v>
       </c>
       <c r="B560" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C560">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="561" spans="1:3" x14ac:dyDescent="0.25">
@@ -7031,15 +7034,15 @@
         <v>721005</v>
       </c>
       <c r="B561" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C561">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="562" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A562">
-        <v>721008</v>
+        <v>721005</v>
       </c>
       <c r="B562" s="1" t="s">
         <v>1</v>
@@ -7050,24 +7053,24 @@
     </row>
     <row r="563" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A563">
+        <v>721008</v>
+      </c>
+      <c r="B563" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C563">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="564" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A564">
         <v>721014</v>
       </c>
-      <c r="B563" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C563">
+      <c r="B564" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C564">
         <v>50</v>
-      </c>
-    </row>
-    <row r="564" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A564" t="s">
-        <v>152</v>
-      </c>
-      <c r="B564" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C564">
-        <v>110</v>
       </c>
     </row>
     <row r="565" spans="1:3" x14ac:dyDescent="0.25">
@@ -7075,32 +7078,32 @@
         <v>152</v>
       </c>
       <c r="B565" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C565">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="566" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A566" t="s">
+        <v>152</v>
+      </c>
+      <c r="B566" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C566">
         <v>60</v>
       </c>
     </row>
-    <row r="566" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A566">
+    <row r="567" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A567">
         <v>241040</v>
       </c>
-      <c r="B566" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C566">
+      <c r="B567" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C567">
         <v>120</v>
-      </c>
-    </row>
-    <row r="567" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A567">
-        <v>241020</v>
-      </c>
-      <c r="B567" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C567">
-        <v>70</v>
       </c>
     </row>
     <row r="568" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7108,43 +7111,43 @@
         <v>241020</v>
       </c>
       <c r="B568" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C568">
-        <v>110</v>
+        <v>70</v>
       </c>
     </row>
     <row r="569" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A569">
-        <v>241040</v>
+        <v>241020</v>
       </c>
       <c r="B569" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C569">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="570" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A570">
-        <v>601138</v>
+        <v>241040</v>
       </c>
       <c r="B570" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C570">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="571" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A571">
-        <v>601128</v>
+        <v>601138</v>
       </c>
       <c r="B571" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C571">
-        <v>80</v>
+        <v>110</v>
       </c>
     </row>
     <row r="572" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7152,54 +7155,54 @@
         <v>601128</v>
       </c>
       <c r="B572" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C572">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="573" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A573">
+        <v>601128</v>
+      </c>
+      <c r="B573" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C573">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="574" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A574">
         <v>601138</v>
       </c>
-      <c r="B573" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C573">
+      <c r="B574" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C574">
         <v>60</v>
-      </c>
-    </row>
-    <row r="574" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A574" t="s">
-        <v>153</v>
-      </c>
-      <c r="B574" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C574">
-        <v>120</v>
       </c>
     </row>
     <row r="575" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A575" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B575" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C575">
-        <v>70</v>
+        <v>120</v>
       </c>
     </row>
     <row r="576" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A576" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B576" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C576">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="577" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7207,31 +7210,42 @@
         <v>155</v>
       </c>
       <c r="B577" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C577">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="578" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A578" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B578" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C578">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="579" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A579" t="s">
+        <v>154</v>
+      </c>
+      <c r="B579" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C579">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="580" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A580" t="s">
         <v>153</v>
       </c>
-      <c r="B579" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C579">
+      <c r="B580" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C580">
         <v>50</v>
       </c>
     </row>

</xml_diff>